<commit_message>
chore(auditoria): actualizar excel con post 50 publicado exitosamente
</commit_message>
<xml_diff>
--- a/auditoria_datos_hde.xlsx
+++ b/auditoria_datos_hde.xlsx
@@ -1122,9 +1122,9 @@
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore(auditoria): sincronizar excel con post 8 publicado
</commit_message>
<xml_diff>
--- a/auditoria_datos_hde.xlsx
+++ b/auditoria_datos_hde.xlsx
@@ -1204,9 +1204,9 @@
       <c r="A9" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore(auditoria): sincronizar excel con post 9 publicado
</commit_message>
<xml_diff>
--- a/auditoria_datos_hde.xlsx
+++ b/auditoria_datos_hde.xlsx
@@ -1286,9 +1286,9 @@
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">

</xml_diff>

<commit_message>
refactor(captions): estandarizar CTA de YouTube en la heladera sin promesas de videos especificos
</commit_message>
<xml_diff>
--- a/auditoria_datos_hde.xlsx
+++ b/auditoria_datos_hde.xlsx
@@ -1434,7 +1434,7 @@
           <t>En plena Gran Depresión, el vicepresidente Julio A. Roca (hijo) firmó en Londres el tratado de comercio con Walter Runciman para asegurar las exportaciones de carne enfriada británicas.
 A cambio, Argentina concedió exenciones aduaneras, trato preferencial al carbón inglés y el monopolio de transporte en Buenos Aires, generando un encendido debate sobre la soberanía económica.
 ¿Conocías los detalles de este pacto? Te leemos en comentarios.
-📺 Mirá el documental sobre la Década Infame en YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #RocaRunciman #HistoriaArgentina #ComercioExterior #CarneArgentina #Economia</t>
         </is>
       </c>
@@ -1516,7 +1516,7 @@
           <t>Mediante la Ley 12.155 se fundó el Banco Central de la República Argentina, con Raúl Prebisch como su primer director general.
 En su origen, el capital estaba compuesto mitad por el Estado y mitad por bancos privados nacionales y extranjeros, con la misión de regular el crédito y la moneda nacional tras el colapso de la Caja de Conversión.
 ¿Sabías que el BCRA no nació 100% estatal? Contanos qué opinás.
-📺 Conocé la historia de las reformas monetarias en YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #BCRA #BancoCentral #RaulPrebisch #HistoriaMonetaria #EconomiaArgentina</t>
         </is>
       </c>
@@ -1598,7 +1598,7 @@
           <t>El exceso de deuda externa tomada por el gobierno de Juárez Celman provocó una crisis financiera colosal en 1890. El Banco Baring Brothers de Londres estuvo al borde de la quiebra total.
 La crisis desembocó en el estallido armado de la Revolución del Parque, la renuncia presidencial y un plan de austeridad histórico encabezado por Carlos Pellegrini.
 ¿Sabías que este default cambió las finanzas mundiales? Te leemos.
-📺 Suscribite a nuestro canal de YouTube: @hablemosdeeco para más historia económica.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #BaringCrisis #CarlosPellegrini #HistoriaArgentina #Default #Economia</t>
         </is>
       </c>
@@ -1680,7 +1680,7 @@
           <t>Durante el gobierno de Onganía y bajo la gestión del ministro Krieger Vasena, entró en vigor el Peso Ley 18.188, reemplazando al Peso Moneda Nacional creado en 1881.
 Fue la primera de varias amputaciones de ceros que sufriría el signo monetario argentino a lo largo del siglo XX a causa del proceso inflacionario crónico.
 ¿Llegaste a usar los billetes del Peso Ley? Compartí tu anécdota.
-📺 Repasamos la historia de todas las monedas argentinas en YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #PesoLey #MonedaArgentina #Numismatica #HistoriaEconomica #Inflacion</t>
         </is>
       </c>
@@ -1762,7 +1762,7 @@
           <t>Hacia el final del régimen militar y con una inflación anual que rozaba el 400%, el Decreto Ley 22.707 creó el Peso Argentino ($a).
 Fue la moneda con menor vida útil de la historia nacional: duró apenas dos años hasta ser reemplazada por el Austral en junio de 1985.
 ¿Por qué creés que ninguna moneda dura en el país? Dejanos tu comentario.
-📺 Conocé la evolución de la inflación argentina en YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #PesoArgentino #HistoriaFinanciera #EconomiaArgentina #Austral #Inflacion</t>
         </is>
       </c>
@@ -1844,7 +1844,7 @@
           <t>El gobierno de Alfonsín intentó revivir la estabilidad con el Plan Primavera: desdoblamiento del mercado cambiario (comercial y financiero), acuerdo de precios con la UIA y alza de tasas de interés.
 Sin embargo, la falta de apoyo del FMI y el drenaje constante de divisas provocó su quiebre en febrero de 1989, dando paso a la primera hiperinflación.
 ¿Recordás los apagones y la crisis de fines del 88? Te leemos.
-📺 Crónica de la hiperinflación de 1989 en YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #PlanPrimavera #Alfonsin #Hiperinflacion #EconomiaArgentina #HistoriaPolitica</t>
         </is>
       </c>
@@ -1926,7 +1926,7 @@
           <t>Aquel lunes de febrero de 1989, el Banco Central suspendió la intervención cambiaria al agotarse sus reservas internacionales operativas.
 El precio del dólar se disparó sin techo, provocando remarcaciones automáticas diarias de precios, desabastecimiento en góndolas y la renuncia anticipada de Raúl Alfonsín meses más tarde.
 ¿Cómo se vivía el día a día remarcando precios? Contanos en los comentarios.
-📺 Más videos históricos en YouTube: @hablemosdeeco (enlace en bio).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #Hiperinflacion1989 #DolarBlue #BCRA #CrisisEconomica #ArgentinaHistorica</t>
         </is>
       </c>
@@ -2008,7 +2008,7 @@
           <t>La Nación y las provincias firmaron el primer Pacto Fiscal para garantizar el equilibrio presupuestario de la Convertibilidad y sostener el déficit de la seguridad social.
 Este acuerdo sentó las bases de los conflictos tributarios federales y la postergada ley de coparticipación ordenada por la Constitución de 1994 que aún sigue pendiente.
 ¿Te parece justo el sistema actual de coparticipación? Dejá tu postura.
-📺 Análisis tributario federal en nuestro canal de YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #PactoFiscal #Coparticipacion #ImpuestosArgentina #EconomiaArgentina #Federalismo</t>
         </is>
       </c>
@@ -2090,7 +2090,7 @@
           <t>Bajo la presidencia de Menem se promulgó la Ley 24.241 que creó las Administradoras de Fondos de Jubilaciones y Pensiones (AFJP).
 Los trabajadores podían elegir entre el reparto estatal y cuentas de ahorro individual administradas por bancos y compañías financieras, sistema que rigió hasta su reestatización en 2008.
 ¿Reparto estatal o capitalización individual? ¿Qué preferís? Te leemos.
-📺 Suscribite a YouTube para análisis económicos completos: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #AFJP #Jubilaciones #SistemaPrevisional #EconomiaArgentina #HistoriaEconomica</t>
         </is>
       </c>
@@ -2172,7 +2172,7 @@
           <t>Tras la devaluación del peso mexicano a fines de 1994, una ola de desconfianza azotó a los mercados emergentes. En Argentina, la convertibilidad enfrentó su primera gran prueba de fuego.
 Cerraron decenas de bancos cooperativos y provinciales, y el gobierno debió crear fondos fiduciarios de rescate para evitar el derrumbe de la paridad 1 a 1.
 ¿Recordás la caída de bancos durante el Tequila? Comentá abajo.
-📺 Mirá el video sobre las corridas bancarias argentinas en YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #EfectoTequila #BancosArgentinos #Convertibilidad #HistoriaEconomica #Finanzas</t>
         </is>
       </c>
@@ -2254,7 +2254,7 @@
           <t>El presidente Fernando de la Rúa anunció por cadena nacional el blindaje financiero con el objetivo de calmar el riesgo país y refinanciar vencimientos de deuda externa.
 A cambio de los fondos, el gobierno se comprometió al déficit cero y al congelamiento del gasto primario, pero la recesión económica no dio tregua.
 ¿Por qué falló el Blindaje financiero? Dejanos tu hipótesis.
-📺 Informe completo del 2000 al 2001 en YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #ElBlindaje #DeLaRua #FMI #DeudaPublica #HistoriaArgentina</t>
         </is>
       </c>
@@ -2336,7 +2336,7 @@
           <t>Conducido por Domingo Cavallo y David Mulford, el Megacanje buscó oxígeno financiero pateando vencimientos de deuda a cambio de tasas de interés de hasta el 16% anual en dólares.
 El alivio de corto plazo incrementó el stock total de deuda, provocando investigaciones judiciales y profundizando el camino hacia el default de diciembre de ese año.
 ¿Era evitable el desenlace del 2001? Te leemos en comentarios.
-📺 Más historia y datos en nuestro YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #Megacanje #DeudaArgentina #Cavallo #Crisis2001 #EconomiaNacional</t>
         </is>
       </c>
@@ -2418,7 +2418,7 @@
           <t>En su discurso inaugural ante la Asamblea Legislativa, el presidente interino Adolfo Rodríguez Saá anunció la suspensión de pagos de la deuda externa soberana ante la ovación de los legisladores.
 Fue el mayor default de la historia moderna hasta ese momento, marginando a la Argentina del crédito voluntario internacional durante más de una década.
 ¿Cómo recordás aquel anuncio en el Congreso? Compartí tu experiencia.
-📺 Seguí nuestros análisis económicos en YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #Default2001 #RodriguezSaa #HistoriaArgentina #DeudaExterna #CrisisEconomica</t>
         </is>
       </c>
@@ -2500,7 +2500,7 @@
           <t>Ante la falta total de liquidez en pesos tras la caída de la convertibilidad, el gobierno bonaerense y otras 14 provincias emitieron bonos para pagar sueldos públicos: Patacones, Lecop, Quebrachos y Federales.
 Los comercios los aceptaban con descuento y cotizaban en pizarras paralelas hasta que fueron rescatados por el gobierno nacional a fines de 2003.
 ¿Llegaste a cobrar o pagar con Patacones? ¿Qué te compraste? Contanos.
-📺 Encontrá el especial sobre cuasimonedas en YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #Patacones #Cuasimonedas #Crisis2002 #Lecop #HistoriaMonetaria</t>
         </is>
       </c>
@@ -2582,7 +2582,7 @@
           <t>El ministro Roberto Lavagna y el secretario Guillermo Nielsen lanzaron la oferta de reestructuración para salir del default de 2001. La aceptación alcanzó el 76% entre los tenedores de bonos.
 Quienes no aceptaron la oferta (los 'holdouts') iniciaron juicios internacionales en Nueva York que derivarían en el recordado conflicto de los Fondos Buitre.
 ¿Considerás que el canje 2005 fue exitoso? Dejá tu opinión en comentarios.
-📺 Suscribite a nuestro canal de YouTube: @hablemosdeeco (link en perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #CanjeDeDeuda #RobertoLavagna #DeudaSoberana #EconomiaArgentina #Holdouts</t>
         </is>
       </c>
@@ -2664,7 +2664,7 @@
           <t>Bajo la presidencia de Néstor Kirchner, Argentina saldó toda su deuda pendiente con el Fondo Monetario Internacional en un único pago en efectivo.
 El objetivo político y económico fue ganar autonomía en la toma de decisiones macroeconómicas sin auditorías periódicas del organismo, emulando la medida tomada por Brasil días antes.
 ¿Fue acertado quemar reservas para cancelar con el FMI? Comentá abajo.
-📺 Mirá el análisis detallado del ciclo 2003-2007 en YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #Kirchner #FMI #ReservasBCRA #HistoriaEconomica #EconomiaArgentina</t>
         </is>
       </c>
@@ -2746,7 +2746,7 @@
           <t>Con el arribo de interventores afines a la Secretaría de Comercio de Guillermo Moreno, se modificó la metodología de medición del Índice de Precios al Consumidor (IPC).
 La brecha entre la inflación oficial y las mediciones privadas superó los 15 puntos porcentuales anuales, afectando los bonos atados a inflación (CER) y las negociaciones paritarias.
 ¿Cómo afectó a tus finanzas la distorsión del IPC? Te leemos.
-📺 Seguí a @hablemosdeeco en YouTube para más informes económicos exclusivos.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #INDEC #Inflacion #GuillermoMoreno #Estadistica #EconomiaArgentina</t>
         </is>
       </c>
@@ -2828,7 +2828,7 @@
           <t>El ministro de Economía Martín Lousteau firmó la Resolución 125 para fijar alícuotas móviles a la exportación de granos según su cotización internacional.
 La medida desató un paro agropecuario histórico de más de 100 días, cortes de ruta y un conflicto político que culminó con el recordado voto 'no positivo' del vicepresidente Julio Cobos.
 ¿Estuviste a favor o en contra de la 125? Dejá tu testimonio.
-📺 Conocé los números del conflicto del campo en YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #Resolucion125 #CampoArgentino #Retenciones #Soja #HistoriaArgentina</t>
         </is>
       </c>
@@ -2910,7 +2910,7 @@
           <t>En medio de la crisis financiera global subprime, el Congreso sancionó la estatización del sistema previsional privado, dando fin a 14 años de régimen de capitalización.
 La ANSES pasó a administrar las carteras de acciones que las AFJP tenían en empresas líderes del país, obteniendo representación en sus directorios.
 ¿Estás a favor del sistema jubilatorio estatal? Debatamos en comentarios.
-📺 Informes de economía e historia en nuestro canal de YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #ANSES #FGS #AFJP #EconomiaArgentina #HistoriaFinanciera</t>
         </is>
       </c>
@@ -2992,7 +2992,7 @@
           <t>Apenas días después de la reelección de Cristina Fernández de Kirchner, se implementó el Programa de Consulta de Operaciones Cambiarias para frenar el drenaje de reservas.
 La medida dio origen a la brecha cambiaria moderna, al resurgimiento del mercado informal ('dólar blue') y a restricciones a las compras con tarjeta en el exterior.
 ¿Recordás cuánto cotizaba el dólar blue en 2011? (Pista: menos de 5 pesos). Te leemos.
-📺 Más contenido sobre la historia del dólar en YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #CepoCambiario #DolarBlue #AFIP #BrechaCambiaria #EconomiaNacional</t>
         </is>
       </c>
@@ -3074,7 +3074,7 @@
           <t>El gobierno nacional anunció la expropiación de las acciones de Repsol en YPF bajo el argumento del vaciamiento de reservas hidrocarburíferas y la pérdida del autoabastecimiento energético.
 La estatización derivó en un acuerdo indemnizatorio con Repsol en 2014 y un litigio multimillonario en tribunales de Nueva York con fondos demandantes que continúa hoy.
 ¿Considerás que YPF debe ser estatal o privada? Justificá tu voto.
-📺 Análisis completo del caso YPF en YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #YPF #VacaMuerta #Petroleo #SoberaniaEnergetica #HistoriaEconomica</t>
         </is>
       </c>
@@ -3156,7 +3156,7 @@
           <t>Bajo la gestión del ministro Axel Kicillof y Juan Carlos Fábrega en el BCRA, el gobierno convalidó un salto del 18% en el tipo de cambio oficial para frenar la sangría de divisas.
 Fue la devaluación más marcada desde 2002, e inauguró el recargo del 35% a cuenta de Ganancias y el cupo mensual para compra de dólar ahorro.
 ¿Cómo impactó esa devaluación en tu día a día? Contanos en los comentarios.
-📺 Conocé más datos monetarios en nuestro YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #Kicillof #Devaluacion #DolarAhorro #BCRA #EconomiaArgentina</t>
         </is>
       </c>
@@ -3238,7 +3238,7 @@
           <t>El juez Thomas Griesa de Nueva York ordenó que Argentina debía pagar 1.330 millones de dólares en efectivo a fondos litigantes (NML Capital) al mismo tiempo que pagaba a bonistas del canje.
 La negativa a pagar desencadenó el denominado 'default técnico' o 'Griesafest', trabando pagos internacionales en el Bank of New York.
 ¿Qué opinás del accionar de los fondos holdouts? Te leemos en comentarios.
-📺 Suscribite a @hablemosdeeco en YouTube para entender los juicios de deuda externa.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #FondosBuitre #Griesa #Holdouts #DeudaExterna #FinanzasInternacionales</t>
         </is>
       </c>
@@ -3320,7 +3320,7 @@
           <t>A una semana de asumir la presidencia de Mauricio Macri, el ministro Alfonso Prat-Gay anunció el levantamiento de las restricciones cambiarias impuestas en 2011.
 El dólar saltó de 9,80 a 13,90 pesos, pero la brecha cambiaria desapareció transitoriamente gracias a un préstamo repo de bancos internacionales para fortalecer reservas.
 ¿Recordás ese día? ¿Pensaste que el dólar se iba más alto? Contanos.
-📺 Mirá el video sobre los ciclos de unificación cambiaria en YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #FinDelCepo #PratGay #DolarHoy #UnificacionCambiaria #EconomiaNacional</t>
         </is>
       </c>
@@ -3402,7 +3402,7 @@
           <t>El ministro de Finanzas Luis Caputo colocó un bono soberano a un siglo de plazo en los mercados internacionales, un instrumento inédito en la historia de la deuda latinoamericana.
 El bono despertó elogios por el plazo extendido de financiamiento pero duras críticas por la tasa convalidada, siendo luego reestructurado en el canje de 2020.
 ¿Emisiones a 100 años: audacia financiera o error estratégico? Dejá tu comentario.
-📺 Más informes sobre deuda soberana en YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #Bono100Años #LuisCaputo #DeudaPublica #MercadoDeCapitales #Economia</t>
         </is>
       </c>
@@ -3484,7 +3484,7 @@
           <t>Tras la corrida cambiaria que disparó el dólar de 20 a 25 pesos y cortó el crédito voluntario de Wall Street, el presidente Macri anunció negociaciones con Christine Lagarde en el FMI.
 Fue el mayor crédito en la historia del organismo multilateral, condicionado a un duro ajuste del déficit fiscal primario.
 ¿Por qué creés que Argentina recurre cíclicamente al Fondo? Te leemos.
-📺 Mirá el especial del acuerdo FMI 2018 en YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #FMI #MauricioMacri #AcuerdoFMI #EconomiaArgentina #HistoriaPolitica</t>
         </is>
       </c>
@@ -3566,7 +3566,7 @@
           <t>Tras el resultado de las PASO de 2019 y la disparada del dólar a 60 pesos, el nuevo ministro Hernán Lacunza anunció la extensión forzosa de los vencimientos de deuda de corto plazo.
 Fue la primera vez que se postergaba compulsivamente el pago de títulos de deuda nominados en moneda local (pesos) en la historia democrática reciente.
 ¿Tenías ahorros en fondos comunes o Letes en ese momento? Contanos.
-📺 Más análisis en nuestro canal de YouTube: @hablemosdeeco (enlace en perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #Reperfilamiento #Lacunza #Letes #Lecaps #EconomiaArgentina</t>
         </is>
       </c>
@@ -3648,7 +3648,7 @@
           <t>Mediante el DNU 596/2019, y tras una pérdida de 3.000 millones de dólares de reservas en dos semanas, el gobierno fijó un tope inicial de 10.000 dólares mensuales, que luego se redujo drásticamente a 200 dólares.
 Esta medida marcó el regreso definitivo de los controles cambiarios que continuarían durante los gobiernos posteriores.
 ¿Creés que algún día Argentina podrá vivir sin cepo cambiario? Te leemos.
-📺 Suscribite a nuestro YouTube: @hablemosdeeco para no perderte ningún análisis.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #CepoCambiario #Dolar200 #ReservasBCRA #HistoriaEconomica #FinanzasPersonales</t>
         </is>
       </c>
@@ -3730,7 +3730,7 @@
           <t>En plena cuarentena por la pandemia de COVID-19, el ministro Martín Guzmán anunció el cierre del acuerdo con los comités de acreedores privados liderados por BlackRock.
 El acuerdo redujo cupones de interés del 7% al 3% anual promedio, aunque no logró bajar el riesgo país de forma sostenible en los años subsiguientes.
 ¿Por qué el riesgo país no bajó tras el canje? Dejá tu lectura económica.
-📺 Análisis profundo del canje Guzmán en YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #MartinGuzman #CanjeDeDeuda #BlackRock #DeudaExterna #EconomiaNacional</t>
         </is>
       </c>
@@ -3812,7 +3812,7 @@
           <t>El Banco Central y la AFIP endurecieron el control de cambios imponiendo una percepción del 35% a cuenta de Ganancias sobre consumos en dólares.
 Además, obligaron a las empresas privadas a refinanciar el 60% de sus deudas financieras en el exterior al restringirles el acceso al Mercado Único y Libre de Cambios.
 ¿Cuánto pagás de impuestos por servicios del exterior hoy? Comentá abajo.
-📺 Seguí a @hablemosdeeco en YouTube para enterarte de todo el archivo económico.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #Supercepo #ImpuestoPais #DolarTarjeta #EconomiaArgentina #AFIP</t>
         </is>
       </c>
@@ -3894,7 +3894,7 @@
           <t>Mientras la vicepresidenta Cristina Kirchner encabezaba un acto en Ensenada, el ministro Guzmán presentó su renuncia indeclinable por redes sociales.
 La incertidumbre política desató corridas en los bonos en pesos, la designación fugaz de Silvina Batakis por 24 días y el salto del dólar informal de 239 a más de 330 pesos.
 ¿Dónde estabas cuando renunció Guzmán? Compartí tu experiencia.
-📺 Más historias económicas en YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #RenunciaGuzman #CrisisPolitica #DolarBlue #EconomiaArgentina #HistoriaReciente</t>
         </is>
       </c>
@@ -3976,7 +3976,7 @@
           <t>Para recomponer las reservas netas negativas del BCRA, el nuevo ministro de Economía Sergio Massa lanzó el Programa de Incremento Exportador.
 El mecanismo permitió al agro liquidar con una cotización superior al dólar oficial, pero implicó una fuerte emisión monetaria por la diferencia pagada por el Banco Central.
 ¿Fue una solución temporal o una trampa de emisión? Dejanos tu postura.
-📺 Mirá el video sobre los tipos de cambio múltiples en YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #DolarSoja #SergioMassa #BCRA #Reservas #EconomiaArgentina</t>
         </is>
       </c>
@@ -4058,7 +4058,7 @@
           <t>El ministro Luis Caputo anunció un paquete de 10 medidas de emergencia económica que incluyó una devaluación del 118%, recorte de subsidios energéticos y suspensión de la obra pública.
 El objetivo central fue alcanzar el superávit fiscal y financiero primario inmediato ('déficit cero') para erradicar la emisión monetaria del BCRA.
 ¿Cómo evalúas el impacto del shock económico? Debatamos con respeto.
-📺 Análisis económico y datos en nuestro YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #JavierMilei #Caputo #DeficitCero #Devaluacion #EconomiaArgentina</t>
         </is>
       </c>
@@ -4140,7 +4140,7 @@
           <t>Bajo la dictadura de Onganía, el ministro Adalbert Krieger Vasena implementó un plan heterodoxo: devaluó el peso pero retuvo parte de la ganancia exportadora para el fisco, congeló salarios y bajó aranceles.
 Logró llevar la inflación al 7% anual en 1969 y atraer inversiones de capital, hasta que el estallido social del 'Cordobazo' puso fin a su gestión.
 ¿Conocías la figura de Krieger Vasena? Te leemos en los comentarios.
-📺 Toda la historia económica la encontrás en YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #KriegerVasena #Cordobazo #HistoriaArgentina #Estabilidad #Economia</t>
         </is>
       </c>
@@ -4222,7 +4222,7 @@
           <t>En un mensaje por radio, el ministro Álvaro Alsogaray acuñó su célebre frase advirtiendo que la sociedad debía soportar meses de sacrificios salariales y tarifazos para sanear las cuentas públicas.
 El plan incluyó eliminación de controles de precios, despido de empleados estatales y emisión de bonos de deuda interna para pagar sueldos atrasados.
 ¿Por qué esa frase sigue tan vigente en Argentina 60 años después? Comentá.
-📺 Más joyas del archivo económico en YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #Alsogaray #HayQuePasarElInvierno #Frondizi #FMI #HistoriaNacional</t>
         </is>
       </c>
@@ -4304,7 +4304,7 @@
           <t>Tras la salida de la crisis de 1890, el presidente Julio A. Roca y su aliado Carlos Pellegrini sancionaron la Ley 3.871, que ató el papel moneda argentino al patrón oro internacional.
 Este régimen monetario rígido garantizó una estabilidad cambiaria casi ininterrumpida durante las tres décadas de mayor crecimiento del modelo agroexportador.
 ¿Sabías que la Convertibilidad existió 90 años antes de Cavallo? Te leemos.
-📺 Documentales completos en nuestro YouTube: @hablemosdeeco (link en perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #PatronOro #CarlosPellegrini #CajaDeConversion #HistoriaEconomica #MonedaNacional</t>
         </is>
       </c>
@@ -4386,7 +4386,7 @@
           <t>Mediante el Decreto 8.503/46 impulsado por el Banco Central bajo la influencia de Miguel Miranda, se eliminó la participación privada en el directorio de la entidad monetaria.
 Además, se estatizaron los depósitos: los bancos operaban como mandatarios del BCRA, reorientando el crédito masivo hacia la industrialización por sustitución de importaciones.
 ¿Bancos públicos o privados para orientar el crédito? ¿Qué opinás? Comentá.
-📺 Todo sobre el peronismo económico en YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #NacionalizacionBCRA #MiguelMiranda #Peronismo #HistoriaFinanciera #Economia</t>
         </is>
       </c>
@@ -4468,7 +4468,7 @@
           <t>En un masivo acto popular en Retiro, Juan Domingo Perón formalizó la adquisición de las líneas férreas británicas utilizando saldos comerciales acumulados durante la Segunda Guerra Mundial.
 La operación garantizó el control nacional de la red de transporte terrestre, aunque abrió debates sobre el precio pagado por material rodante desgastado.
 ¿Fue una gesta de soberanía o un pésimo negocio financiero? Dejá tu punto de vista.
-📺 Documentales sobre transporte y economía en YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #FerrocarrilesArgentinos #Nacionalizacion #Peron #HistoriaArgentina #Economia</t>
         </is>
       </c>
@@ -4550,7 +4550,7 @@
           <t>El segundo mandato de Perón comenzó con un viraje económico: el Plan Económico de 1952 implementó austeridad fiscal, congelamiento de precios y salarios por dos años y un día sin carne por semana.
 El plan logró frenar la inflación del 50% al 4% anual en 1954 y reorientó incentivos de inversión hacia el agro y la energía con la firma de contratos petroleros.
 ¿Conocías el giro ortodoxo de Perón en 1952? Comentanos qué te parece.
-📺 Mirá el video completo sobre el Plan 1952 en YouTube: @hablemosdeeco.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #PlanEconomico1952 #Peron #HistoriaEconomica #Inflacion #Austeridad</t>
         </is>
       </c>
@@ -4632,7 +4632,7 @@
           <t>El presidente Arturo Frondizi anunció por cadena nacional la apertura al capital privado internacional para exploración y explotación de hidrocarburos a través de YPF.
 La producción de petróleo se triplicó en apenas 36 meses, eliminando la sangría de dólares por importación de combustibles, pese a la feroz oposición política de la época.
 ¿Desarrollismo o dependencia? ¿Qué opinás de la política de Frondizi? Te leemos.
-📺 Suscribite a nuestro canal de YouTube: @hablemosdeeco para más debates históricos.
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #Frondizi #BatallaDelPetroleo #YPF #Desarrollismo #HistoriaNacional</t>
         </is>
       </c>
@@ -4796,7 +4796,7 @@
           <t>Apenas asumió el gobierno de la Alianza, el ministro José Luis Machinea impulsó la 'Tablita de Machinea', subiendo las alícuotas del impuesto a las ganancias y recortando deducciones a sueldos medios y altos.
 Lejos de sanear las cuentas, la medida deprimió el consumo interno y profundizó la recesión que desembocaría en la crisis terminal de 2001.
 ¿Sufriste el impacto de la Tablita de Machinea en tu salario? Te leemos.
-📺 Más historias económicas argentinas en YouTube: @hablemosdeeco (enlace en perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #Machinea #Impuestazo #LaAlianza #Ganancias #HistoriaEconomica</t>
         </is>
       </c>
@@ -4878,7 +4878,7 @@
           <t>El 30 de noviembre de 2001 el sistema financiero argentino vivió su jornada más negra. En apenas veinticuatro horas, ahorristas y corporaciones retiraron más de 1.000 millones de dólares ante el rumor inminente de una devaluación y la negativa del FMI a girar fondos frescos.
 Esa sangría descontrolada elevó la pérdida mensual de depósitos a casi 4.000 millones de dólares y dejó las reservas del Banco Central en un piso crítico. Sin margen de maniobra, el ministro Domingo Cavallo y Fernando de la Rúa firmaron a medianoche el Decreto 1570, congelando el dinero de millones de argentinos.
 ¿Recordás el clima en las calles los días previos a la firma del Corralito? Te leemos en comentarios.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -4960,7 +4960,7 @@
           <t>En julio de 2001, con el riesgo país superando los 1.600 puntos básicos y los mercados internacionales cerrados, el gobierno de Fernando de la Rúa impulsó la desesperada Ley de Déficit Cero. El Estado se comprometía por ley a no gastar un solo peso más de lo que ingresaba por recaudación.
 La variable de ajuste fue inmediata y despiadada: un recorte automático del 13% en los haberes de empleados públicos y en jubilaciones que superaban los 500 pesos. Lejos de calmar a los inversores, la medida contrajo el consumo interno, profundizó la recesión y destruyó la recaudación fiscal.
 ¿Creés que el Déficit Cero pudo haber evitado el estallido si se aplicaba antes? Dejanos tu opinión.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -5042,7 +5042,7 @@
           <t>La implosión de la Convertibilidad y la megadevaluación de 2002 pulverizaron el tejido social argentino. La medición del INDEC de mayo de 2002 arrojó una desocupación abierta del 21,5%, el registro oficial más alto en la historia moderna del país.
 Más de dos millones y medio de personas quedaron sin trabajo formal y la pobreza subió a un dramático 53%. El salario real se derrumbó cerca de un 30% en meses y la economía argentina acumuló una contracción per cápita del 28% entre 1998 y 2002.
 ¿Cómo vivió tu familia o tu entorno aquel durísimo año 2002? Te leemos en comentarios.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -5124,7 +5124,7 @@
           <t>En febrero de 2002, el presidente Eduardo Duhalde y el ministro Jorge Remes Lenicov firmaron el Decreto 214/2002, consagrando la polémica 'pesificación asimétrica'. La medida buscó evitar la quiebra masiva de deudores bancarios pero destrozó el balance de las entidades financieras.
 Los préstamos hipotecarios y comerciales se convirtieron a pesos a razón de uno a uno ($1 por dólar), mientras que los depósitos atrapados en los bancos se pesificaron a $1,40 ajustados por inflación (CER). La diferencia patrimonial multimillonaria fue asumida por el Estado emitiendo deuda pública.
 ¿Fue la pesificación asimétrica un rescate necesario o una transferencia ilegítima? Opiná abajo.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -5206,7 +5206,7 @@
           <t>Julio de 1989 quedó grabado como el mes más destructivo en la historia monetaria argentina. Con el Plan Austral y el Plan Primavera completamente destruidos, los precios se remarcaban dos o tres veces en un mismo día y los comercios cerraban por desabastecimiento.
 La inflación mensual rozó el 200% y la moneda nacional perdió toda función de reserva. La crisis forzó a Raúl Alfonsín a entregar el mando presidencial a Carlos Menem cinco meses antes de lo estipulado por la Constitución, en medio de saqueos y estado de sitio.
 ¿Tenés anécdotas familiares sobre cómo se cobraba el sueldo en plena hiper del 89? Contanos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -5288,7 +5288,7 @@
           <t>Al recuperar la democracia en 1983, el gobierno de Raúl Alfonsín se topó con un corset financiero letal: la última dictadura militar había sextuplicado la deuda externa, elevándola de 8.000 a más de 45.000 millones de dólares.
 El ministro Bernardo Grinspun intentó liderar un club de deudores latinoamericanos para negociar en bloque, pero la Reserva Federal de EE.UU. mantenía tasas de interés por encima del 15% anual. El pago de intereses consumía más de la mitad de las divisas que generaba el campo argentino.
 ¿Pensás que Alfonsín debió haber desconocido la deuda externa de la dictadura? Debatamos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -5370,7 +5370,7 @@
           <t>La relación entre el gobierno alfonsinista y la Confederación General del Trabajo (CGT) fue una guerra de desgaste constante. Encabezada por el cervecero Saúl Ubaldini, la central obrera desplegó una ofensiva sindical sin precedentes: 13 paros generales en cinco años y medio.
 Bajo el lema de romper con el FMI y congelar tarifas, las protestas debilitaron los anclajes de precios de Juan Vital Sourrouille y complicaron la aprobación de leyes clave en el Congreso, acelerando el desgaste del gobierno hacia el final de su mandato.
 ¿Fueron reclamos genuinos por la pérdida salarial o una embestida política del peronismo? Te leemos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -5452,7 +5452,7 @@
           <t>A fines de marzo de 1989, tras el colapso del Plan Primavera y la renuncia de Juan Vital Sourrouille, Raúl Alfonsín convocó a un veterano dirigente radical para intentar calmar a los mercados: Juan Carlos Pugliese. La corrida contra el austral era incontenible.
 Tras reunirse con banqueros, exportadores y formadores de precios pidiéndoles tregua, Pugliese brindó una conferencia de prensa histórica donde admitió con desazón: 'Les hablé con el corazón y me respondieron con el bolsillo'. Pocas semanas después dejaba su cargo.
 ¿Puede la política frenar una corrida cambiaria apelando a la buena voluntad? Dejanos tu postura.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -5534,7 +5534,7 @@
           <t>En mayo de 1946, Juan Domingo Perón creó el Instituto Argentino de Promoción del Intercambio (IAPI), estatizando el comercio exterior de granos y carnes. En un mundo devastado por la Segunda Guerra Mundial, Argentina concentraba gran parte de los alimentos que Europa necesitaba con urgencia.
 El mecanismo era directo: el IAPI pagaba un precio fijo en pesos a los chacareros locales y vendía la cosecha a precios internacionales exorbitantes en divisas. Con esa gigantesca masa de recursos, el gobierno subsidió el crédito industrial y congeló los alimentos en las ciudades.
 ¿Fue el IAPI un motor de industrialización necesario o el inicio de la asfixia del campo? Opiná abajo.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -5616,7 +5616,7 @@
           <t>El Instituto Argentino de Promoción del Intercambio (IAPI), fundado en 1946 como monopolio del comercio exterior, mostró sus límites estructurales hacia 1952. Tras años de transferir renta del campo a la industria, el desplome de las cosechas y de los precios mundiales desató pérdidas colosales.
 Para cubrir el quebranto comercial, el Banco Central debió emitir moneda sin respaldo por el equivalente al 15% del Producto Bruto Interno, forzando a Perón a lanzar su Plan Económico de Emergencia y congelar precios.
 ¿Pudo sostenerse en el tiempo el monopolio estatal del comercio exterior? Te leemos en comentarios.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -5698,7 +5698,7 @@
           <t>Durante la Segunda Guerra Mundial, Gran Bretaña financió sus compras masivas de carne y granos argentinos mediante libras esterlinas que quedaron congeladas en el Banco de Inglaterra por la inconvertibilidad posbélica.
 Ante el riesgo cierto de que esas 150 millones de libras sufrieran una devaluación o repudio formal en Londres, el gobierno argentino optó por destinarlas a la compra de las cuatro compañías ferroviarias británicas.
 ¿Fue una compra estratégica de soberanía o una salida obligada ante el bloqueo británico? Comentá tu postura.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -5780,7 +5780,7 @@
           <t>La entrega de ENTel en noviembre de 1990 fue el mascarón de proa del plan de privatizaciones de Carlos Menem. Conseguir una línea fija estatal demoraba hasta diez años y las denuncias por corrupción y desidia eran moneda corriente en los hogares argentinos.
 Para seducir a Telefónica de España y al consorcio de Telecom, la interventora María Julia Alsogaray aplicó aumentos tarifarios previos de hasta un 300% y garantizó contratos de exclusividad monopólica por una década, transformando el déficit estatal en tarifas dolarizadas.
 ¿Creés que las privatizaciones mejoraron los servicios o crearon monopolios privados? Te leemos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -5862,7 +5862,7 @@
           <t>El 14 de mayo de 1995, Carlos Menem obtuvo la reelección presidencial en primera vuelta con casi el 50% de los votos. Sin embargo, en paralelo a la estabilidad del peso convertible, la economía sufría un shock demoledor por la crisis mexicana del Tequila.
 Ese mismo mes, el INDEC midió una desocupación del 18,4%, la más alta registrada hasta ese momento. La falta de flexibilidad cambiaria de la Convertibilidad obligaba a ajustar vía salarios y destrucción de empleo masivo en el sector productivo.
 ¿Por qué creés que la sociedad votó masivamente por la continuidad a pesar del desempleo? Comentá.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -5944,7 +5944,7 @@
           <t>Fundada por Hipólito Yrigoyen y Enrique Mosconi en 1922, YPF era el buque insignia de las empresas públicas argentinas. Tras décadas de administración estatal deficitaria, en junio de 1993 el gobierno de Carlos Menem llevó a cabo una oferta pública inicial histórica en Wall Street.
 La venta de acciones recaudó más de 3.000 millones de dólares que se destinaron a pagar deudas previsionales con jubilados y sanear las cuentas fiscales. Seis años más tarde, la española Repsol adquiriría el control total de la petrolera.
 ¿Hizo bien el país en privatizar YPF en los 90 o fue un error estratégico? Dejanos tu postura.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -6026,7 +6026,7 @@
           <t>En noviembre de 1989, frente a las huelgas del gremio ferroviario 'La Fraternidad', Carlos Menem pronunció una de sus frases más recordadas: 'Ramal que para, ramal que cierra'. Ferrocarriles Argentinos perdía en ese momento más de un millón de dólares diarios.
 El plan de concesiones y clausuras desmanteló casi el 75% de la red de pasajeros del interior del país, aislando a cientos de pueblos y concentrando el transporte de cargas en camiones por rutas provinciales y nacionales.
 ¿Qué impacto tuvo la pérdida del ferrocarril en el interior productivo del país? Comentá abajo.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -6108,7 +6108,7 @@
           <t>A fines del siglo XIX, la inserción de Argentina en la división internacional del trabajo convirtió al país en una potencia agroexportadora global. Los puertos del Río de la Plata despachaban millones de toneladas de trigo, maíz y carne congelada hacia una Europa industrializada.
 Las estadísticas históricas demuestran que hacia 1895 el PBI per cápita argentino duplicaba al de Italia o España y superaba a naciones como Francia o Alemania. Sin embargo, la riqueza estaba fuertemente concentrada y carecía de una base industrial propia.
 ¿Era un modelo sostenible en el tiempo o condenado al agotamiento? Dejanos tu postura.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -6190,7 +6190,7 @@
           <t>Argentina y Australia compartían a comienzos del siglo XX una dotación de recursos similar: inmensas extensiones de tierra fértil, baja densidad poblacional y fuerte inmigración europea. Ambas colonias alimentaban al Imperio Británico.
 La ruptura comenzó tras la Segunda Guerra Mundial: mientras Australia mantuvo moneda sana, seguridad jurídica y diversificó sus exportaciones mineras e industriales, Argentina cayó en una espiral de inflación crónica, cepos y golpes de Estado que erosionaron el capital productivo.
 ¿Cuál fue el factor determinante del atraso argentino frente a Australia? Te leemos en el debate.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -6272,7 +6272,7 @@
           <t>El crecimiento económico vertiginoso de la Argentina de fines del siglo XIX y principios del XX descansó en la continua anexión de hectáreas fértiles y la expansión de la red de trenes. Pero hacia 1930 la frontera pampeana llegó a su límite físico.
 La caída de la productividad marginal de la tierra, sumada al crac de Wall Street de 1929 y el cierre de mercados internacionales, provocó el colapso de las exportaciones y forzó el inicio de la Industrialización por Sustitución de Importaciones (ISI).
 ¿Pudo Argentina haber continuado viviendo exclusivamente del campo después de 1930? Opiná.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -6354,7 +6354,7 @@
           <t>La reforma previsional de 1994 impulsada por Domingo Cavallo creó las AFJP, privatizando una parte sustancial de los aportes jubilatorios. El Estado dejó de percibir los aportes de los trabajadores en blanco pero debió seguir pagando las jubilaciones de los adultos mayores en curso.
 El sistema privado cobraba comisiones leoninas: hasta un 35% de los aportes se diluía en costos de administración y seguros de vida antes de invertirse. Además, las administradoras prestaban gran parte de ese dinero al propio Estado mediante bonos soberanos.
 ¿Fue el sistema de capitalización privada una estafa o un ahorro arruinado por el Estado? Te leemos en comentarios.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -6436,7 +6436,7 @@
           <t>Al disolver las AFJP y promulgar la Ley 26.425 en diciembre de 2008, el Estado nacional no solo absorbió bonos públicos, sino también carteras millonarias de acciones en empresas privadas que las AFJP habían comprado con los aportes de los trabajadores.
 El Estado nacional se convirtió de la noche a la mañana en accionista de Techint, Telecom, Grupo Clarín, Banco Macro y Siderar, designando directores estatales en sus asambleas y cobrando dividendos multimillonarios que nutrieron el Fondo de Garantía de Sustentabilidad.
 ¿Estuvo bien que el Estado tomara asiento en los directorios de grandes empresas? Comentá abajo.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -6518,7 +6518,7 @@
           <t>En septiembre de 2008, la quiebra del banco de inversión Lehman Brothers desató el pánico bursátil en todo el mundo. En Argentina, las AFJP tenían una porción sustancial de sus carteras invertida en acciones locales y fondos internacionales atados a Wall Street.
 El desplome evaporó cerca del 20% del valor patrimonial de los ahorros previsionales en cuestión de semanas. El argumento del desplome global fue el catalizador político que utilizó Amado Boudou para convencer a la presidenta de estatizar de urgencia el sistema.
 ¿La crisis de 2008 justificaba la estatización o se usó como pretexto político? Te leemos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -6600,7 +6600,7 @@
           <t>En febrero de 2011, la Secretaría de Comercio Interior intensificó la persecución penal y multas de hasta 500.000 pesos contra consultoras económicas privadas que difundían mediciones de inflación superiores a las del INDEC intervenido.
 Para romper el cerco de censura, legisladores de diversos bloques de la oposición crearon el 'IPC Congreso', utilizando sus fueros parlamentarios para publicar mensualmente el promedio de las estimaciones privadas y visibilizar la suba real del costo de vida.
 ¿Recordás el impacto que generaba el IPC Congreso cada mes? Te leemos en comentarios.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -6682,7 +6682,7 @@
           <t>A comienzos de 2011, la brecha entre la inflación oficial del INDEC (cercana al 9% anual) y la inflación real de los supermercados (que superaba el 25%) era insostenible. Ante esta situación, el gobierno aplicó la Ley de Lealtad Comercial para multar con medio millón de pesos a las consultoras que medían precios.
 La persecución judicial obligó a los diputados de la oposición a unificar los datos privados y difundir mensualmente el 'IPC Congreso' desde el recinto para eludir las sanciones y la censura del Poder Ejecutivo.
 ¿Recordás la época en que la inflación real era un tabú sancionado por el Estado? Te leemos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -6764,7 +6764,7 @@
           <t>Las consecuencias de manipular las estadísticas del INDEC no fueron gratis. Durante el canje de deuda de 2005, Argentina había emitido 'Cupones PBI', un instrumento que pagaba un premio a los bonistas si el país crecía por encima del 3,2% anual.
 En 2014, el ministro Axel Kicillof modificó el año base del cálculo estadístico de 1993 a 2004, reduciendo retroactivamente el crecimiento declarado para no gatillar el pago de 3.000 millones de dólares. Los fondos internacionales demandaron al país y ganaron el juicio en los tribunales de Londres.
 ¿Ahorró plata el Estado o terminó pagando el triple por alterar los números? Comentá abajo.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -6846,7 +6846,7 @@
           <t>Hacia el final del mandato de Alberto Fernández y la gestión de Sergio Massa, el Banco Central recurrió a una emisión masiva de Letras de Liquidez (Leliqs) y Pases pasivos para retirar de circulación los billones de pesos emitidos durante la pandemia y el 'Plan Platita'.
 El stock de deuda remunerada alcanzó la friolera de 30 billones de pesos, devengando intereses diarios equivalentes a miles de millones de pesos. La masa de pasivos amenazaba con derivar en una hiperinflación si no se desactivaba de urgencia.
 ¿Fue la bola de Leliqs la bomba económica más peligrosa recibida en 2023? Opiná en los comentarios.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -6928,7 +6928,7 @@
           <t>Para evitar devaluar el tipo de cambio oficial sin reservas líquidas, el Ministerio de Economía implementó en 2022 el Sistema de Importaciones de la República Argentina (SIRA). Las empresas debían importar insumos financiándose con sus propios proveedores en el exterior a 180 días.
 Al postergarse los pagos mes a mes, la deuda comercial privada acumulada superó los 50.000 millones de dólares en diciembre de 2023, paralizando líneas de producción automotriz, farmacéutica e insumos básicos por falta de pago a casas matrices extranjeras.
 ¿Conocías la magnitud oculta de la deuda comercial de las SIRA? Compartí tu experiencia.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -7010,7 +7010,7 @@
           <t>El balance del Banco Central al finalizar 2023 exhibió el deterioro patrimonial más severo desde la hiperinflación de 1989. Aunque las reservas brutas figuraban en 21.000 millones de dólares, restando los pasivos exigibles el saldo neto era de 11.000 millones de dólares en rojo.
 Para intervenir en los dólares financieros y pagar importaciones de energía en invierno, la autoridad monetaria consumió los dólares del swap con el Banco Popular de China e incluso recurrió transitoriamente a la liquidez de los encajes bancarios privados.
 ¿Cómo logró la economía argentina funcionar sin reservas netas durante meses? Te leemos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -7092,7 +7092,7 @@
           <t>En julio de 1944, 44 países aliados se reunieron en Bretton Woods para diseñar la arquitectura financiera de la posguerra. John Maynard Keynes advirtió que atar el comercio mundial a la moneda nacional de una sola potencia generaría desequilibrios globales permanentes.
 Keynes propuso el 'Bancor', una unidad de cuenta administrada por una Unión de Compensación que multaría tanto a los países con déficit crónico como a los que acumulaban superávit comercial. Sin embargo, la supremacía militar y económica de EE.UU. impuso al dólar convertible en oro.
 ¿Habría sido más estable la economía mundial con el Bancor de Keynes? Dejanos tu postura.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -7174,7 +7174,7 @@
           <t>Durante décadas, la ortodoxia keynesiana descansó sobre la 'Curva de Phillips': la creencia de que un gobierno podía reducir el desempleo tolerando una inflación un poco más alta. El shock petrolero de la OPEP en 1973 destruyó ese dogma por completo.
 El precio del crudo se cuadruplicó y las economías occidentales experimentaron inflación de dos dígitos con desempleo masivo simultáneo (estanflación). Economistas como Milton Friedman y Friedrich Hayek cobraron protagonismo al demostrar que la emisión solo compra ilusión a corto plazo.
 ¿Creés que la inflación genera actividad económica o destruye el salario real? Comentá abajo.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -7256,7 +7256,7 @@
           <t>Frente al desempleo masivo de la Gran Depresión de los años 30, el economista británico John Maynard Keynes publicó su 'Teoría General del Empleo, el Interés y el Dinero', que revolucionó la ciencia económica moderna.
 Keynes desafió la ley clásica de Say: argumentó que los salarios a la baja deprimen el consumo y que el Estado debe endeudarse o emitir para financiar obras públicas. Su concepto del 'multiplicador' postuló que cada peso inyectado por el fisco genera más de un peso de ingreso nacional.
 ¿El gasto público rescata a la economía o genera deuda e inflación futura? Queremos saber tu opinión.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -7338,7 +7338,7 @@
           <t>El sueño de la casa propia se transformó en una quimera para las nuevas generaciones en Argentina. El encarecimiento relativo del metro cuadrado dolarizado sumado al desplome histórico de los salarios reales en moneda dura pulverizó el acceso a la vivienda.
 Mientras en la década del 90 un trabajador formal calificado podía adquirir un metro cuadrado de construcción con dos sueldos, en la actualidad la cifra asciende a seis remuneraciones íntegras sin gastar un solo peso en comida ni servicios.
 ¿Cuánto tiempo le llevaría a un joven comprar una vivienda con el salario actual? Te leemos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -7420,7 +7420,7 @@
           <t>En junio de 2020, con amplio consenso parlamentario, se sancionó la Ley de Alquileres 27.551 buscando proteger a los inquilinos. La norma extendió el plazo mínimo a tres años y prohibió cualquier ajuste que no fuera anual mediante el índice ICL del Banco Central.
 En un contexto de inflación desbocada superior al 100%, el resultado fue catastrófico: los propietarios retiraron sus departamentos del mercado, los precios iniciales aumentaron un 300% para cubrirse de la licuación y florecieron los contratos ilegales en dólares.
 ¿Fue la Ley de Alquileres la regulación económica más perjudicial de los últimos años? Opiná.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -7502,7 +7502,7 @@
           <t>En 2016, el Banco Central presidido por Federico Sturzenegger lanzó la Unidad de Valor Adquisitivo (UVA), inspirada en el modelo chileno de las UF. La cuota inicial se calculaba a tasas bajas en pesos y se indexaba mensualmente por el índice de precios al consumidor.
 Durante dos años se vivió un boom de escrituras y más de 100.000 familias accedieron a su primera vivienda. Sin embargo, cuando la inflación saltó del 25% al 50% y luego al 100% mientras los sueldos se rezagaban, la cuota devoró una porción creciente de los ingresos familiares.
 ¿Fueron los créditos UVA una gran oportunidad o una trampa indexada? Contanos tu experiencia.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -7584,7 +7584,7 @@
           <t>El marco regulatorio que rige la explotación de litio, oro y cobre en Argentina fue diseñado en 1993 bajo el gobierno de Carlos Menem. La Ley 24.196 garantizó a las multinacionales mineras estabilidad tributaria absoluta por tres décadas.
 Además, la legislación estableció que las provincias (dueñas originarias de los recursos naturales según la Constitución) no pueden cobrar más del 3% de regalías sobre el valor mineral extraído en boca de mina, dejando el grueso de la renta en manos de los operadores globales.
 ¿Deberían modificarse las regalías del litio para financiar escuelas y hospitales? Debatamos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -7666,7 +7666,7 @@
           <t>Uno de los discursos más repetidos en la política argentina es la exigencia de fabricar baterías de autos eléctricos a escala masiva en las provincias del norte. Sin embargo, la química de almacenamiento revela una realidad técnica muy diferente.
 El litio es apenas el ingrediente menor de una celda moderna: requiere níquel refinado de Indonesia, cobalto de África, grafito sintético de China y nanotecnología de precisión que insumen miles de millones de dólares. Argentina produce la materia prima básica pero carece de la cadena industrial.
 ¿Tiene sentido exportar el mineral purificado o el Estado debe forzar la industrialización local? Contanos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -7748,7 +7748,7 @@
           <t>En la puna andina compartida por Argentina, Bolivia y Chile se encuentra el mayor reservorio de salmuera de litio del planeta. A diferencia de Australia, que extrae litio de roca dura mediante minería tradicional altamente costosa, los salares sudamericanos utilizan evaporación solar natural.
 Sin embargo, los tres países aplicaron modelos antagónicos: Chile fijó regalías progresivas de hasta el 40%, Bolivia estatizó el recurso paralizando la producción y Argentina apostó a concesiones privadas con bajas regalías pero rápida radicación de inversiones.
 ¿Cuál de los tres modelos de explotación del litio considerás más exitoso? Opiná en comentarios.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -7830,7 +7830,7 @@
           <t>En 1919, el inmigrante italiano Carlos Ponzi descubrió una falla en el sistema postal internacional: los cupones de respuesta comprados en una Europa devaluada por la guerra podían canjearse por estampillas en EE.UU. a un valor nominal más alto.
 Ponzi montó una estructura financiera prometiendo ganancias siderales en semanas. Pero el arbitraje era impracticable a gran escala: Ponzi simplemente utilizaba el dinero de los nuevos ahorristas para pagar intereses a los viejos, hasta que el esquema implosionó en agosto de 1920.
 ¿Por qué creés que la gente sigue cayendo en esquemas piramidales un siglo después? Te leemos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -7912,7 +7912,7 @@
           <t>A comienzos de 2022 estalló el mayor fraude piramidal de la era digital argentina: Generación Zoe. Encabezada por Leonardo Cositorto, la organización combinaba discursos de coaching ontológico, teología de la prosperidad y finanzas descentralizadas.
 Prometían retornos fijos del 7,5% mensual en dólares y la compra de un token propio respaldado en supuestos lingotes de oro. Cuando la entrada de nuevos aportantes no alcanzó para cubrir los retiros, los directivos huyeron del país y la justicia dictó órdenes de captura internacional.
 ¿Llegaste a conocer a alguien que haya invertido en Generación Zoe o esquemas similares? Comentá.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -7994,7 +7994,7 @@
           <t>Durante años, Enrique Blaksley Señorans fue el símbolo del éxito financiero en la alta sociedad porteña. A través del fondo Hope Funds, patrocinaba eventos con Roger Federer, Usain Bolt y el club La Dolfina de polo, atrayendo ahorros con contratos de mutuo que prometían intereses del 12% anual en dólares.
 La fachada se derrumbó cuando se descubrió que los fondos eran desviados a sociedades en Panamá e Islas Vírgenes para comprar mansiones y campos. En 2023 la justicia federal lo condenó por liderar una de las mayores estafas piramidales de la historia del país.
 ¿Qué rol juega el marketing de lujo en la credibilidad de estos esquemas fraudulentos? Opiná.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -8076,7 +8076,7 @@
           <t>En abril de 2020, bajo el argumento de la crisis sanitaria por COVID-19, el Comité Ejecutivo de la AFA comandado por Claudio Tapia tomó una decisión inédita: anular los descensos de categoría en el fútbol argentino por dos temporadas completas.
 Lejos de ser una medida excepcional, la abolición del castigo deportivo se extendió y consolidó un torneo hipertrofiado de casi 30 equipos en Primera División. La pérdida de competitividad devaluó los derechos internacionales de transmisión frente al poderío del Brasileirao.
 ¿El formato actual protege a los clubes con problemas financieros o destruye el nivel del fútbol? Opiná.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -8158,7 +8158,7 @@
           <t>Detrás de la gloria deportiva obtenida por la Scaloneta en Qatar 2022, la Asociación del Fútbol Argentino enfrenta un complejo frente judicial en los tribunales federales de Comodoro Py. Denuncias por lavado de activos, contratos con firmas offshore y presuntas irregularidades fiscales.
 Investigaciones periodísticas revelaron que contratos clave de sponsoreo internacional y venta de entradas fueron cedidos a empresas intermediarias creadas en Miami y Delaware, reduciendo los ingresos directos que debían percibir los clubes afiliados a la AFA.
 ¿Por qué los éxitos de la Selección tapan las sospechas de corrupción dirigencial? Dejanos tu punto de vista.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -8240,7 +8240,7 @@
           <t>En agosto de 2009, en medio de una asfixia financiera de los clubes y un paro de Futbolistas Argentinos Agremiados, Julio Humberto Grondona rompió unilateralmente el vínculo de exclusividad televisiva con Torneos y Competencias y el Grupo Clarín.
 El Estado nacional asumió la transmisión gratuita a través del programa 'Fútbol para Todos', estatizando las pautas publicitarias con propaganda oficial. La iniciativa absorbió miles de millones de pesos del presupuesto nacional hasta su cancelación definitiva en 2017.
 ¿Fue una conquista social del acceso al deporte o un despilfarro de fondos públicos? Debatamos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -8322,7 +8322,7 @@
           <t>El 30 de junio de 2021, la Legislatura de Tierra del Fuego aprobó por unanimidad una ley histórica que prohibió la instalación de granjas de cultivo de salmónidos en las aguas del Canal Beagle. La medida fue impulsada por organizaciones ecologistas que alertaron sobre el uso de antibióticos y daño a los fondos marinos.
 La decisión convirtió a la provincia en pionera global de protección ambiental, pero clausuró una industria acuícola que podría haber generado miles de empleos calificados y divisas por exportación en una provincia dependiente del subsidio fiscal industrial.
 ¿Priorizás la preservación ecológica absoluta o la explotación productiva sustentable? Te leemos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -8404,7 +8404,7 @@
           <t>Las aguas frías y prístinas del Cono Sur representan un ecosistema privilegiado para la cría de salmón. Sin embargo, las políticas de ambos lados de la cordillera tomaron caminos radicalmente opuestos.
 Mientras Argentina vetó la actividad en el Canal Beagle, Chile desarrolló en sus fiordos una industria que exporta más de 6.000 millones de dólares anuales a Estados Unidos, Japón y Brasil, convirtiéndose en el segundo exportador mundial y generando empleo formal en regiones australes aisladas.
 ¿Debería Argentina revisar la prohibición adoptando estándares noruegos modernos? Dejanos tu postura.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -8486,7 +8486,7 @@
           <t>A pesar de la disputa de soberanía argentina, el gobierno británico de las Islas Malvinas construyó su prosperidad financiera vendiendo permisos de pesca en aguas disputadas del Atlántico Sur a flotas de España, Taiwán y Corea del Sur.
 La venta de licencias de calamar Illex y merluza negra genera decenas de millones de libras esterlinas al año, transformando a los 3.000 habitantes isleños en una de las poblaciones con mayor ingreso per cápita del mundo gracias a los recursos marítimos argentinos.
 ¿Cómo debería defender Argentina sus recursos pesqueros en la plataforma continental? Te leemos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -8568,7 +8568,7 @@
           <t>Creado por el general Charles de Gaulle en 1945, el Franco CFA (Comunidad Financiera Africana) sigue rigiendo el destino económico de catorce países de África Central y Occidental. A pesar de haber obtenido la independencia política en los años 60, su soberanía monetaria permanece atada a París.
 Francia garantiza la paridad cambiaria fija de la moneda con el euro, pero a cambio obligó durante décadas a los bancos centrales africanos a depositar la mitad de sus reservas internacionales directamente en una cuenta operativa del Tesoro francés.
 ¿Es el Franco CFA un ancla de estabilidad para África o una herramienta de dominio colonial? Opiná.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -8650,7 +8650,7 @@
           <t>Francia se presenta ante el mundo como el líder indiscutido de la energía nuclear limpia en Europa. Gran parte del mineral radiactivo que alimenta sus 56 reactores atómicos provino históricamente de las minas explotadas por la estatal Orano en Níger.
 La paradoja del desarrollo es abrumadora: mientras las luces de París y la industria francesa funcionan con uranio nigerino, más del 80% de la población de Níger vive en la oscuridad más absoluta sin acceso a tendido eléctrico ni agua potable.
 ¿Conocías el trasfondo de recursos detrás del poder nuclear europeo? Te leemos en comentarios.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -8732,7 +8732,7 @@
           <t>En enero de 1994, ante la pérdida de competitividad de las exportaciones africanas y la presión del FMI, el primer ministro francés Édouard Balladur decidió unilateralmente una devaluación del 50% del Franco CFA respecto al franco francés.
 De la noche a la mañana, millones de familias en Senegal, Costa de Marfil, Malí y Camerún vieron duplicarse el precio en moneda local del arroz, la harina y los medicamentos importados, desatando revueltas sociales y desmintiendo la supuesta autonomía africana.
 ¿Puede una nación ser verdaderamente libre si no maneja su propio banco central? Dejanos tu postura.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -8814,7 +8814,7 @@
           <t>El informe de pobreza del INDEC publicado en septiembre de 2024 expuso la peor crisis social registrada en el Norte Grande argentino. En el aglomerado urbano de Gran Resistencia (Chaco), tres de cada cuatro habitantes no alcanzaron a cubrir la canasta básica total.
 La falta de industrias privadas, la destrucción del poder de compra salarial y una economía informal que supera el 50% convirtieron a la capital chaqueña en el epicentro de la indigencia, a pesar de décadas de transferencias discrecionales y coparticipación federal.
 ¿Por qué el asistencialismo no logró reducir la pobreza estructural en el Norte? Dejanos tu opinión.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -8896,7 +8896,7 @@
           <t>Concordia, la segunda ciudad de Entre Ríos, representa uno de los enigmas económicos más dolorosos del país. Ubicada sobre la rica cuenca del río Uruguay y sede de la represa hidroeléctrica de Salto Grande, compite año tras año por el primer puesto de pobreza urbana del INDEC.
 La causa estructural reside en la informalidad: miles de familias dependen del 'trabajo golondrina' durante las cosechas de cítricos y arándanos, quedando sin ingresos durante los meses de invierno y dependiendo de programas de asistencia municipal y provincial.
 ¿Cómo se explica tanta pobreza en una de las zonas productivas más fértiles del Litoral? Comentá.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -8978,7 +8978,7 @@
           <t>La asimetría del mercado laboral argentino se evidencia con crudeza al cruzar la General Paz hacia el interior profundo. En varias provincias del norte argentino, el empleo público provincial y municipal se transformó en la única red de contención económica ante la ausencia de inversión privada.
 Estadísticas del Ministerio de Trabajo demuestran que en provincias como Formosa existen más de 160 empleados públicos por cada 100 trabajadores formales del sector privado, financiados mediante el reparto de la coparticipación federal que tributan las provincias pampeanas.
 ¿Es viable el desarrollo de un país con provincias donde el Estado supera al sector privado? Opiná.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -9060,7 +9060,7 @@
           <t>En junio de 1930, en un intento desesperado por proteger a los agricultores e industrias norteamericanas tras el crac de Wall Street, el presidente Herbert Hoover promulgó la Ley Arancelaria Smoot-Hawley, subiendo aranceles a más de 20.000 productos importados.
 La respuesta internacional fue inmediata: Europa, Canadá y América Latina cerraron sus fronteras comerciales. En apenas tres años, el volumen del comercio mundial se contrajo dos tercios y la desocupación se disparó, enseñando al mundo los peligros del proteccionismo a ultranza.
 ¿Creés que las guerras comerciales protegen a los trabajadores locales o empobrecen a todos? Te leemos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -9142,7 +9142,7 @@
           <t>Durante la primera presidencia de Donald Trump, las industrias argentinas de valor agregado sufrieron un golpe devastador. En agosto de 2017, la Comisión de Comercio Internacional de EE.UU. falló a favor de los 'farmers' norteamericanos y acusó a Argentina de subsidiar el biodiésel de soja.
 EE.UU. aplicó aranceles punitivos de más del 70%, cerrando de la noche a la mañana el principal destino de exportación del polo aceitero del Gran Rosario, que generaba más de 1.200 millones de dólares anuales para la balanza comercial argentina.
 ¿El proteccionismo de las potencias es el mayor obstáculo para la industria argentina? Dejanos tu visión.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -9224,7 +9224,7 @@
           <t>En marzo de 2018, Donald Trump invocó la histórica Sección 232 de la Ley de Expansión Comercial de 1962 para imponer aranceles globales del 25% a las importaciones de acero y del 10% al aluminio, alegando proteger la base industrial bélica de los Estados Unidos.
 La medida puso en jaque a las plantas siderúrgicas de Aluar en Puerto Madryn y de Tenaris (Techint) en Campana. Solo tras intensas gestiones diplomáticas, Argentina logró negociar cuotas de exportación libres de arancel a cambio de limitar sus envíos anuales.
 ¿Puede un país emergente negociar de igual a igual frente a gigantes proteccionistas? Opiná abajo.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -9306,7 +9306,7 @@
           <t>La sanción de la Ley Bases 27.742 consagró la aprobación del Régimen de Incentivo para Grandes Inversiones (RIGI). El esquema busca destrabar megaproyectos en minería de litio y cobre, gasoductos de GNL en Vaca Muerta y plantas de energía renovable.
 A cambio de hundir un mínimo de 200 millones de dólares, el Estado garantiza estabilidad fiscal por tres décadas, reducción de alícuotas del impuesto a las ganancias y la libre disponibilidad de divisas de exportación sin obligación de liquidar en el Banco Central.
 ¿Considerás que el RIGI atraerá inversiones reales o regala soberanía tributaria? Opiná abajo.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -9388,7 +9388,7 @@
           <t>En agosto de 2023, durante la cumbre de Johannesburgo, el gobierno de Alberto Fernández había celebrado la invitación para que Argentina ingrese formalmente a los BRICS a partir del 1 de enero de 2024 junto a potencias como Arabia Saudita, Irán y Emiratos Árabes.
 Apenas tres semanas después de asumir, Javier Milei remitió notas oficiales a Lula da Silva, Xi Jinping y Vladimir Putin declinando la membresía y ratificando el alineamiento geopolítico irrestricto de Argentina con Estados Unidos e Israel.
 ¿Hizo bien Argentina en bajarse de los BRICS o desaprovechó un mercado emergente clave? Debatamos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -9470,7 +9470,7 @@
           <t>A pesar de la retórica confrontativa durante la campaña electoral, la realidad de las reservas líquidas forzó un pragmatismo diplomático ineludible. En junio de 2024, el Banco Central de la República Argentina logró renovar el tramo de libre disponibilidad del swap de monedas con China.
 Eran 35.000 millones de yuanes (equivalentes a 5.000 millones de dólares) que vencían en el corto plazo y hubieran provocado un default técnico de no refinanciarse, demostrando el peso ineludible de Beijing en las finanzas del país.
 ¿Puede Argentina desligarse comercialmente de China en el mundo actual? Dejanos tu postura.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -9552,7 +9552,7 @@
           <t>Buscando disputar la hegemonía crediticia global que el Fondo Monetario Internacional y el Banco Mundial ostentan desde 1944, los mandatarios de Brasil, Rusia, India, China y Sudáfrica fundaron en 2014 el Nuevo Banco de Desarrollo (NBD), con sede central en Shanghái.
 El banco fue concebido para financiar carreteras, puertos y represas en economías en desarrollo sin exigirles los tradicionales programas de austeridad y reformas estructurales exigidos por Washington.
 ¿Representa el NBD una alternativa real al FMI para América Latina? Te leemos en comentarios.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -9634,7 +9634,7 @@
           <t>El 5 de agosto de 2024, los mercados financieros globales experimentaron una ola de pánico bautizada como el nuevo 'Lunes Negro'. El detonante ocurrió en Tokio: el Banco de Japón abandonó sus tasas de interés negativas y las subió al 0,25%, apreciando el yen con violencia.
 Esto provocó el cierre apresurado del 'Carry Trade': inversores de todo el mundo que se endeudaban en yenes baratos para comprar acciones tecnológicas y bonos en Wall Street vendieron sus activos en masa para saldar deudas, contagiando a todas las bolsas del planeta.
 ¿Sentiste el impacto de la volatilidad financiera internacional en las criptos o acciones? Te leemos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -9716,7 +9716,7 @@
           <t>Creada por la economista Claudia Sahm, la 'Regla de Sahm' establece que cuando el promedio móvil de tres meses de la tasa de desempleo en EE.UU. sube 0,5 puntos porcentuales respecto de su mínimo del año anterior, la economía ya entró en recesión.
 En agosto de 2024, el reporte laboral norteamericano encendió todas las alarmas al escalar al 4,3%. Los inversores temieron que la Reserva Federal se hubiera demorado en recortar las tasas de interés, asfixiando el crédito productivo y el consumo de los hogares.
 ¿Logrará EE.UU. un aterrizaje suave de su economía o la recesión es inevitable? Opiná abajo.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -9798,7 +9798,7 @@
           <t>En julio de 2024, el Departamento del Tesoro de EE.UU. confirmó un hito sin precedentes: la deuda pública total del gobierno federal superó los 35 billones de dólares, equivalentes a más del 120% de su Producto Bruto Interno.
 Con las tasas de interés en máximos de dos décadas para combatir la inflación de la pospandemia, el gobierno norteamericano debe destinar más de 1 billón de dólares anuales exclusivamente al pago de intereses, superando el gasto del Pentágono en armamento y tropas.
 ¿Podrá Estados Unidos pagar su deuda o terminará licuándola con emisión monetaria? Dejanos tu visión.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -9880,7 +9880,7 @@
           <t>Cada vez que las centrales obreras decretan una huelga general en Argentina, la discusión pública se polariza entre el derecho constitucional a huelga y el daño financiero que causa a la actividad privada. En abril de 2024, la CGT convocó a su segunda medida de fuerza contra la administración de Milei.
 Estudios económicos estiman que un paro total que paralice el transporte público en el AMBA y las terminales agroexportadoras de Rosario le cuesta al país más de 500 millones de dólares diarios en bienes no producidos, fletes demorados y ventas perdidas.
 ¿Considerás que el paro general es una herramienta válida de reclamo o perjudica a la economía? Contanos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -9962,7 +9962,7 @@
           <t>El poder financiero del sindicalismo argentino se apoya en una herramienta legal única: la retención compulsiva en el recibo de sueldo. A través de las cláusulas de 'solidaridad', las empresas descuentan entre el 1% y el 3% del salario bruto de todos los trabajadores encuadrados en convenio, estén o no afiliados al gremio.
 Este flujo ininterrumpido de millones de pesos alimenta las cajas sindicales sin que los trabajadores puedan optar por desvincularse del aporte, un punto que generó fuertes batallas judiciales en los amparos laborales contra el DNU 70/2023.
 ¿Debería ser optativa la cuota sindical para los trabajadores no afiliados? Dejanos tu postura.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -10044,7 +10044,7 @@
           <t>El 24 de enero de 2024, la conducción de la CGT protagonizó una huelga general histórica. Apenas 45 días después de la jura presidencial de Javier Milei, las centrales sindicales movilizaron al Congreso en rechazo al DNU 70/2023 de desregulación económica.
 Fue el paro más temprano convocado a un presidente desde el regreso de la democracia: a Raúl Alfonsín le realizaron su primer paro a los nueve meses de mandato, a Carlos Menem al tercer año y a Mauricio Macri a los dieciséis meses de gobierno.
 ¿Fue una reacción justificada ante el shock económico o una muestra de doble vara gremial? Debatamos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -10126,7 +10126,7 @@
           <t>En diciembre de 2023, la economía argentina experimentó un fogonazo inflacionario histórico tras la corrección del tipo de cambio oficial de 360 a 800 pesos por dólar. El traslado inmediato a precios (pass-through) impulsó el IPC mensual al 25,5%.
 Alimentos y artículos de primera necesidad registraron subas superiores al 30%, licuando drásticamente el poder adquisitivo de salarios y jubilaciones. Sin embargo, el ancla fiscal del déficit cero impidió la espiralización hacia una hiperinflación en los meses siguientes.
 ¿Fue inevitable el impacto del 25,5% para corregir precios reprimidos? Te leemos en comentarios.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -10208,7 +10208,7 @@
           <t>Hacia finales de 2023, el cepo cambiario argentino alcanzó niveles grotescos de complejidad burocrática. Para evitar devaluar el tipo de cambio mayorista sin reservas en el Banco Central, el Palacio de Hacienda inventó tipos de cambio a medida de cada sector productivo y cultural.
 Surgieron el 'Dólar Soja' para incentivar liquidaciones agrarias, el 'Dólar Coldplay' para espectáculos internacionales, el 'Dólar Qatar' con recargos impositivos para turistas y el 'Dólar Malbec'. Esta fragmentación alimentó una masiva sobrefacturación y arbitrajes fraudulentos.
 ¿Cuál fue el tipo de cambio más insólito que recordás de la época del supercepo? Contanos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -10290,7 +10290,7 @@
           <t>Para desactivar la bomba de las deudas comerciales heredadas del sistema SIRA sin entregar dólares inmediatos de las reservas, el Banco Central ideó el Bopreal (Bonos para la Reconstrucción de una Argentina Libre).
 Los importadores suscribieron estos títulos públicos nominados en dólares pagando con sus pesos atrapados en el sistema bancario. Al comercializarse en los mercados secundarios, el bono absorbió billones de pesos de la plaza y permitió normalizar la cadena de suministros industriales.
 ¿Fue el Bopreal una solución técnica brillante o estatizar deuda de empresas privadas? Comentá.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -10372,7 +10372,7 @@
           <t>El ancla del programa económico de 2024 fue el ajuste fiscal más drástico en la historia moderna de Argentina. Por primera vez desde 2008, el Estado nacional acumuló cinco meses consecutivos de superávit fiscal financiero, es decir, gastando menos de lo que recaudó incluso tras abonar los servicios de deuda.
 El resultado se logró mediante una combinación de 'motosierra' y 'licuadora': suspensión total de transferencias no automáticas a provincias, freno absoluto a la obra pública nacional y postergación de la actualización de jubilaciones y salarios estatales.
 ¿Es sostenible el superávit fiscal si no se reactiva la economía y el consumo? Te leemos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -10454,7 +10454,7 @@
           <t>La pérdida de poder adquisitivo del salario formal e informal a lo largo de 2024 provocó una transformación histórica en la mesa de los argentinos. Tradicionalmente el país con mayor consumo de carne vacuna del mundo, la cifra per cápita retrocedió a mínimos que no se veían desde 1914.
 Con un promedio de 44,8 kilos anuales por persona, los consumidores reemplazaron masivamente los cortes vacunos por carne de pollo y cerdo más accesibles, reflejando el impacto de la recesión en el consumo básico familiar.
 ¿Tuviste que recortar o cambiar el consumo de carne en tu hogar durante 2024? Comentá abajo.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -10536,7 +10536,7 @@
           <t>El Régimen de Regularización de Activos impulsado en 2024 superó todas las expectativas iniciales de los analistas financieros. Con alícuota cero para montos de hasta 100.000 dólares y facilidades para fondos mayores que permanecieran en el sistema, los ahorristas blanquearon masivamente divisas 'del colchón'.
 Los depósitos en dólares del sector privado en los bancos argentinos crecieron a niveles que no se registraban desde antes de las elecciones primarias de agosto de 2019, recomponiendo la liquidez del sistema bancario local.
 ¿Creés que los dólares del blanqueo se volcarán a créditos hipotecarios y productivos? Dejanos tu postura.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -10618,7 +10618,7 @@
           <t>A mediados de julio de 2024, el ministro Luis Caputo y el presidente del Banco Central Santiago Bausili ejecutaron la 'Fase 2' del programa monetario: eliminar la emisión endógena por intereses de pasivos remunerados.
 Los bancos comerciales dejaron de colocar su liquidez en pases diarios del Banco Central y migraron sus fondos a Letras de Liquidez Fiscal (Lefi) emitidas directamente por el Tesoro Nacional. De esta forma, el costo del pago de intereses pasó a ser absorbido por el superávit fiscal primario.
 ¿Es mejor que la deuda de los bancos la pague el Tesoro con recaudación en vez de emitir dinero? Opiná.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -10700,7 +10700,7 @@
           <t>Milton Friedman acuñó su célebre máxima: 'La inflación es siempre y en todo lugar un fenómeno monetario'. En Argentina, generaciones de gobernantes intentaron refutarlo aplicando controles de precios, ley de abastecimiento, juntas reguladoras y pactos sociales.
 Sin embargo, cada vez que el Banco Central expandió la cantidad de dinero para financiar el déficit del Tesoro, la inflación reapareció con violencia desmedida. La desaceleración de precios lograda en 2024 tras cerrar la canilla de emisión ratificó una vez más el postulado monetarista.
 ¿Pensás que la emisión es la única causa de la inflación o inciden factores estructurales? Debatamos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -10782,7 +10782,7 @@
           <t>Las elecciones presidenciales de 2023 sepultaron cuarenta años de alternancia política tradicional en Argentina. La grieta entre el peronismo kirchnerista y la coalición de Juntos por el Cambio implosionó ante la emergencia de un outsider libertario sin estructura territorial ni gobernadores propios.
 El colapso del bipartidismo obedeció a un dato material contundente: doce años consecutivos con el PBI per cápita estancado, destrucción del salario en dólares y una inflación que cerró 2023 por encima del 211%, rompiendo la lealtad partidaria de las clases medias y populares.
 ¿Se cerró definitivamente el ciclo de la grieta tradicional en Argentina? Dejanos tu opinión.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -10864,7 +10864,7 @@
           <t>Pocos pueblos en el mundo desarrollaron una gimnasia económica tan sofisticada como los argentinos. Sobrevivir a dos hiperinflaciones, nueve defaults soberanos y la eliminación sucesiva de trece ceros a la moneda moldeó una cultura financiera única en el planeta.
 Desde operar con cotizaciones paralelas y tasas de interés diarias hasta ahorrar en billetes físicos bajo el colchón, el argentino promedio gestiona riesgos financieros que desconcertarían a cualquier economista europeo, manteniendo la pasión e identidad a pesar de las crisis recurrentes.
 ¿Qué aprendizaje económico te transmitieron tus padres o abuelos para sortear las crisis? Te leemos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -10946,7 +10946,7 @@
           <t>En octubre de 2024, el indicador de riesgo país elaborado por JP Morgan perforó la barrera psicológica de los 1.000 puntos básicos. Hacía más de cuatro años, desde la reestructuración de deuda de Martín Guzmán en 2020, que los bonos soberanos argentinos no cotizaban con paridades tan elevadas.
 La compresión de la prima de riesgo reflejó la confianza de los fondos de inversión internacionales en la disciplina fiscal innegociable y la acumulación de reservas vía blanqueo y liquidaciones de exportaciones.
 ¿Alcanza con bajar el riesgo país para que vuelvan las inversiones productivas de gran escala? Te leemos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -11028,7 +11028,7 @@
           <t>Uno de los capítulos más debatidos de la Ley Bases fue la reforma del régimen de indemnizaciones de la Ley de Contrato de Trabajo. El texto facultó a gremios y cámaras empresarias a reemplazar la indemnización tradicional por un Fondo de Cese Laboral financiado mensualmente por el empleador.
 El objetivo declarado es eliminar la litigiosidad y la 'industria del juicio' que frena la contratación formal en pequeñas y medianas empresas, otorgando al trabajador un fondo acumulado al desvincularse, con independencia de la causa de despido.
 ¿El fondo de cese moderniza el mercado laboral o debilita los derechos del trabajador? Comentá.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -11110,7 +11110,7 @@
           <t>El 8 de julio de 1884 el Congreso Nacional sancionó la histórica Ley 1420 de Educación Común, una de las reformas estructurales más trascendentes de la Generación del 80.
 La norma estableció que la escuela primaria debía ser gratuita, obligatoria, gradual y laica. Esta política de Estado transformó el capital humano del país, integrando a millones de hijos de inmigrantes y reduciendo el analfabetismo a niveles comparables con las potencias europeas.
 ¿Fue la educación pública el motor principal del progreso argentino de fines del siglo XIX? Te leemos en comentarios.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -11192,7 +11192,7 @@
           <t>Impulsada por salarios reales que superaban a los de gran parte de Europa y el estímulo constitucional a la inmigración, Argentina experimentó una transformación demográfica única en el mundo.
 Entre 1880 y el estallido de la Primera Guerra Mundial llegaron más de cuatro millones de italianos, españoles y de diversas nacionalidades, proveyendo la fuerza de trabajo que dinamizó la agricultura pampeana y el comercio urbano.
 ¿Cómo moldeó la inmigración masiva la cultura del trabajo y la economía nacional? Te leemos en comentarios.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -11274,7 +11274,7 @@
           <t>En la Exposición Universal de París de 1889, donde se inauguró la Torre Eiffel, la República Argentina deslumbró al mundo con un monumental pabellón de hierro, bronce y vitrales de dos plantas.
 El Estado invirtió sumas récord para exhibir sus granos, carnes, maderas y minerales, posicionándose como una de las economías emergentes más atractivas para las inversiones extranjeras de la época.
 ¿Representó París 1889 el cenit de la inserción de Argentina en el comercio global? Comentá abajo.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -11356,7 +11356,7 @@
           <t>En septiembre de 1907, ante el incremento incesante del costo de vida y los abusos de los propietarios, estalló en los conventillos de San Telmo y La Boca una inédita huelga de pagos.
 Familias enteras de trabajadores organizaron comités barriales para resistir los desalojos policiales y demandar una rebaja del 30% en los alquileres y condiciones sanitarias dignas, marcando un hito en la lucha urbana.
 ¿Es la dificultad para acceder a la vivienda un problema centenario en el país? Te leemos en comentarios.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -11438,7 +11438,7 @@
           <t>Hacia el inicio de la Gran Guerra, el tendido férreo argentino había alcanzado casi 34.000 kilómetros de extensión, permitiendo llevar la producción agropecuaria pampeana hasta los puertos de ultramar en cuestión de horas.
 Construida fundamentalmente con capitales británicos y franceses, junto a líneas estatales de fomento, la red ferroviaria consolidó la integración territorial del modelo agroexportador.
 ¿Fue el tren el gran articulador del despegue productivo nacional? Dejanos tu punto de vista.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -11520,7 +11520,7 @@
           <t>El colapso de la Bolsa de Nueva York en octubre de 1929 y la Gran Depresión posterior golpearon de lleno a la economía argentina, sumamente vulnerable a las fluctuaciones de la demanda mundial.
 El precio de los cereales y la carne se hundió en los mercados internacionales, reduciendo drásticamente las divisas disponibles y precipitando una profunda crisis política y fiscal que derivó en el golpe de 1930.
 ¿Demostró la crisis del 30 el agotamiento del modelo exclusivamente agroexportador? Opiná abajo.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -11602,7 +11602,7 @@
           <t>En octubre de 1931, asediado por la escasez de divisas y la salida incesante de reservas metálicas de la Caja de Conversión, el gobierno argentino implementó el primer control de cambios formal de su historia.
 Se creó la Comisión de Control de Cambios, obligando a los exportadores a liquidar sus divisas al tipo oficial y racionando la venta a los importadores mediante permisos previos de asignación.
 ¿Nacieron allí las raíces de las restricciones cambiarias recurrentes del país? Te leemos en comentarios.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -11684,7 +11684,7 @@
           <t>Ante la brutal caída de la recaudación por aranceles aduaneros generada por el desplome del comercio mundial en la década de 1930, el Estado debió buscar nuevas fuentes de financiamiento interno.
 Así nació el Impuesto a los Réditos (antecesor directo del impuesto a las ganancias), con una alícuota básica inicial del 3%. Aunque se promulgó como una medida de emergencia provisoria por tres años, jamás fue derogado.
 ¿Por qué los impuestos provisionales en Argentina tienden a volverse eternos? Te leemos en comentarios.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -11766,7 +11766,7 @@
           <t>A fines de 1952 el Congreso Nacional aprobó el Segundo Plan Quinquenal, que marcó un giro sustancial respecto a la política de industrialización acelerada y subsidios masivos del primer mandato peronista.
 El plan priorizó la austeridad fiscal, incentivó el aumento de la productividad agropecuaria con mejores precios y buscó captar inversiones extranjeras en petróleo y maquinaria para aliviar el estrangulamiento de la balanza de pagos.
 ¿Fue un ajuste pragmático necesario ante la escasez de reservas? Te leemos en comentarios.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -11848,7 +11848,7 @@
           <t>Consciente del enorme drenaje de divisas que representaba la importación de combustibles, Juan Domingo Perón firmó en 1955 un precontrato con la Standard Oil de California para la explotación de petróleo en la Patagonia.
 La iniciativa contemplaba otorgar amplios derechos de prospección y explotación sobre 40.000 kilómetros cuadrados, generando fuertes críticas de la oposición y de sectores nacionalistas que rechazaban la apertura a firmas foráneas.
 ¿Habría alcanzado Argentina el autoabastecimiento antes con este acuerdo? Comentá abajo.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -11930,7 +11930,7 @@
           <t>Cumpliendo con su principal promesa de campaña electoral, el presidente Arturo Illia anuló mediante decretos los contratos petroleros firmados durante la gestión de Arturo Frondizi con multinacionales petroleras.
 La medida argumentó vicios de procedimiento y defensa de la soberanía de YPF, pero derivó en costosos litigios indemnizatorios internacionales y un freno en la extracción que forzó al país a reanudar la importación de hidrocarburos.
 ¿Fue una decisión de principios soberana o un retroceso productivo? Te leemos en comentarios.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -12012,7 +12012,7 @@
           <t>Impulsada por el ministro de Salud Arturo Oñativia bajo el mandato de Illia, la Ley 16.463 reguló el mercado farmacéutico declarando a los medicamentos bienes sociales.
 La normativa congeló precios, obligó a auditar los costos de producción reales de las drogas y promovió el uso de genéricos, desatando un duro enfrentamiento con laboratorios multinacionales que influyó en el clima previo al golpe militar de 1966.
 ¿Debe el Estado regular estrictamente los precios de los medicamentos esenciales? Dejanos tu visión.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -12094,7 +12094,7 @@
           <t>Apenas restablecida la democracia en diciembre de 1983, el equipo económico de Raúl Alfonsín encaró la reforma de la Dirección General Impositiva (DGI) ante niveles de evasión fiscal que superaban el 50%.
 Se unificaron los registros dispersos de personas y empresas creando la Clave Única de Identificación Tributaria (CUIT), herramienta informática fundacional para cruzar datos bancarios y patrimoniales en la recaudación moderna.
 ¿Alcanzan los cruces informáticos para doblegar la evasión estructural? Te leemos en comentarios.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -12176,7 +12176,7 @@
           <t>El 26 de marzo de 1991 los presidentes de Argentina, Brasil, Paraguay y Uruguay estamparon su firma en el Tratado de Asunción, creando formalmente el Mercado Común del Sur (Mercosur).
 El acuerdo eliminó progresivamente los aranceles entre los países miembros y estableció una política comercial común, convirtiendo a Brasil en el principal socio comercial e industrial de Argentina durante las tres décadas siguientes.
 ¿Ha sido el Mercosur un puente integrador o una traba arancelaria para el país? Te leemos en comentarios.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -12258,7 +12258,7 @@
           <t>Dentro del ambicioso plan de privatizaciones del Estado encabezado por el ministro Roberto Dromi, Aerolíneas Argentinas fue transferida en noviembre de 1990 a un consorcio liderado por la estatal española Iberia.
 La operación contempló una combinación de pago en divisas y entrega de títulos de deuda soberana argentina con fuertes quitas, iniciando un controvertido proceso de desinversión y venta de aeronaves y rutas comerciales.
 ¿Fue la privatización de Aerolíneas un negocio ruinoso para el patrimonio nacional? Comentá abajo.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -12340,7 +12340,7 @@
           <t>Tras meses de ardua negociación parlamentaria donde se excluyeron de la lista a YPF, Banco Nación y Aerolíneas Argentinas, la Ley Bases 27.742 declaró 'sujetas a privatización' o concesión a un conjunto selecto de empresas en manos del Estado nacional.
 Quedaron habilitadas para su venta total o parcial compañías como Energía Argentina S.A. (Enarsa), la prestadora aeroportuaria Intercargo y Agua y Saneamientos Argentinos (AySA), así como la operación privada de las líneas ferroviarias de transporte de granos.
 ¿El Estado debe gestionar empresas de servicios o dejarlas en manos de privados? Queremos saber tu opinión.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -12422,7 +12422,7 @@
           <t>A fines de 1991 el gobierno sancionó la Ley Nacional de Empleo 24.013, que flexibilizó el régimen contractual laboral creando contratos temporales y de pasantía exentos de indemnizaciones.
 Buscando reducir los costos laborales de las empresas y estimular contrataciones en el nuevo contexto de estabilidad monetaria, la flexibilización no logró impedir que el desempleo escalara a dos dígitos hacia mediados de la década.
 ¿Baja el costo laboral el desempleo o fomenta la precariedad? Dejanos tu postura.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -12504,7 +12504,7 @@
           <t>El 28 de diciembre de 1992 culminó el traspaso formal de Gas del Estado, la colosal empresa pública que durante décadas administró la red de gasoductos más importante de América del Sur.
 El sistema fue fragmentado verticalmente en dos transportadoras troncales y ocho distribuidoras regionales, atrayendo a consorcios internacionales y extendiendo la red de gas natural domiciliario a nuevas provincias.
 ¿Fue la privatización del gas un modelo regulatorio exitoso? Te leemos en comentarios.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -12586,7 +12586,7 @@
           <t>Sociedad Mixta Siderúrgica Argentina (Somisa), el mayor complejo de acero integrado del país fundado bajo el impulso del general Manuel Savio, fue privatizada en octubre de 1992.
 La intervención estatal ejecutó un drástico ajuste previo reduciendo la plantilla laboral de 12.000 a menos de 5.000 trabajadores antes de transferir el polo siderúrgico de San Nicolás a Techint, naciendo Siderar.
 ¿Justificaba el déficit de las empresas públicas este tipo de privatizaciones? Comentá abajo.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -12668,7 +12668,7 @@
           <t>Durante el cimbronazo financiero del Efecto Tequila en 1995, el gobierno nacional creó el Fondo Fiduciario para el Desarrollo Provincial (FFDP) con el respaldo de préstamos del Banco Mundial y el BID.
 El fondo aportó liquidez para sanear los abultados quebrantos de los bancos públicos provinciales, condicionando el rescate a su venta o traspaso al sector privado para cortar el déficit cuasifiscal del interior.
 ¿Estuvo bien condicionar el auxilio financiero a la privatización de los bancos? Opiná abajo.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -12750,7 +12750,7 @@
           <t>En agosto de 1998 Rusia devaluó el rublo y declaró la moratoria unilateral sobre sus títulos de deuda soberana, desatando una masiva huida de capitales desde todos los mercados emergentes hacia activos de refugio.
 Para la Argentina de la Convertibilidad, altamente dependiente del financiamiento externo para cubrir su déficit de cuenta corriente, significó un salto abrupto en las tasas de interés y el comienzo de la larga recesión que culminó en 2001.
 ¿Fue el shock ruso el principio del fin para el régimen de tipo de cambio fijo? Te leemos en comentarios.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -12832,7 +12832,7 @@
           <t>Tras la salida traumática de la Convertibilidad en los primeros meses de 2002, el presidente Eduardo Duhalde promulgó el Decreto 214/2002 implementando la polémica 'pesificación asimétrica'.
 Las deudas bancarias de particulares y empresas se convirtieron a un peso por dólar, mientras que los depósitos en dólares de los ahorristas se reconocieron a 1,40 pesos indexados por inflación (CER), provocando un colosal déficit en las entidades.
 ¿Fue la pesificación asimétrica un salvataje a grandes deudores a costa del fisco? Dejanos tu opinión.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -12914,7 +12914,7 @@
           <t>Mediante el Decreto 905/2002, el Estado nacional estructuró la emisión masiva de los Bonos del Gobierno Nacional (Boden 2012 y 2013) para evitar la liquidación judicial del sistema financiero tras el colapso del Corralito.
 Los títulos en moneda extranjera fueron entregados a las entidades bancarias para compensar el descalce patrimonial y a los ahorristas que optaron por canjear sus plazos fijos atrapados, culminando de pagarse diez años después.
 ¿Terminaron todos los contribuyentes pagando el costo del derrumbe bancario? Te leemos en comentarios.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -12996,7 +12996,7 @@
           <t>En abril de 2010 el ministro de Economía Amado Boudou anunció la reapertura de la reestructuración soberana para aquellos bonistas que no habían ingresado en la operación de 2005.
 La oferta ofreció condiciones financieras más duras que la original, pero logró elevar la aceptación global al 92,4% de la deuda defaulteada en 2001, dejando afuera al 7,6% de fondos litigantes que luego triunfarían ante la corte de Nueva York.
 ¿Se debió haber cerrado un acuerdo definitivo con el remanente en ese momento? Comentá abajo.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -13078,7 +13078,7 @@
           <t>A fines de agosto de 2012, en plena vigencia del cepo cambiario y ante la creciente salida de reservas por turismo internacional, la AFIP oficializó la Resolución General 3378.
 Se fijó una percepción a cuenta de Ganancias y Bienes Personales del 15% sobre compras con tarjeta de crédito en el exterior, inaugurando un esquema de tipos de cambio diferenciales para viajes y servicios que perdura hasta hoy.
 ¿Frenan los recargos cambiarios la demanda de dólares o estimulan la brecha informal? Te leemos en comentarios.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -13160,7 +13160,7 @@
           <t>En mayo de 2014 el ministro de Economía Axel Kicillof viajó a Francia y rubricó un entendimiento con las naciones que integran el Club de París para regularizar los pasivos impagos desde la crisis de 2001.
 El acuerdo no requirió el monitoreo tradicional del FMI pero implicó reconocer intereses compensatorios y punitorios acumulados que llevaron el saldo a casi 9.700 millones de dólares con un cronograma de pago a cinco años.
 ¿Fue conveniente convalidar la tasa del 9% para volver a los mercados financieros? Opiná abajo.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -13242,7 +13242,7 @@
           <t>El 21 de marzo de 2006 el gobierno de Néstor Kirchner puso fin por decreto a la concesión de Aguas Argentinas en el Área Metropolitana de Buenos Aires, en manos del consorcio encabezado por la firma francesa Suez.
 El Estado alegó incumplimiento reiterado en las metas de inversión de agua corriente y saneamiento ambiental, creando la empresa pública Agua y Saneamientos Argentinos (AySA) con el 90% de participación estatal.
 ¿Mejoró la gestión del servicio sanitario tras su reestatización? Dejanos tu experiencia.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -13324,7 +13324,7 @@
           <t>En marzo de 2006, buscando contener la suba de precios en los mostradores de las carnicerías urbanas, la Secretaría de Comercio dispuso la suspensión total de las exportaciones de carne vacuna por seis meses.
 La medida provocó la pérdida de mercados internacionales clave ganados durante décadas y un desincentivo ganadero que condujo a la liquidación de más de 12 millones de cabezas de ganado bovino en los años posteriores.
 ¿Logran las prohibiciones a la exportación bajar los precios de forma duradera? Te leemos en comentarios.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -13406,7 +13406,7 @@
           <t>A fines de octubre de 2009, mediante el Decreto de Necesidad y Urgencia 1602/09, el Poder Ejecutivo creó la Asignación Universal por Hijo para Protección Social financiada a través de los recursos de la ANSES.
 El beneficio igualó las asignaciones familiares contributivas para hijos de empleados no registrados, monotributistas sociales y desocupados, condicionando el cobro mensual a la acreditación de escolaridad y controles de vacunación.
 ¿Ha sido la AUH la política de contención social más eficaz contra la indigencia? Comentá tu visión.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -13488,7 +13488,7 @@
           <t>En agosto de 2018, en el marco del programa de aceleración del ajuste fiscal acordado con el FMI, el gobierno de Mauricio Macri derogó el Fondo Federal Solidario creado durante el conflicto del campo en 2009.
 La eliminación del reparto del 30% de los derechos de exportación del complejo sojero generó un duro reclamo de gobernadores e intendentes de todo el país, que utilizaban esos recursos exclusivamente para infraestructura sanitaria y vial.
 ¿Deben las retenciones agropecuarias coparticiparse siempre con las provincias? Te leemos en comentarios.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -13570,7 +13570,7 @@
           <t>El 1 de septiembre de 1992 comenzaron a operar formalmente Edenor y Edesur, compañías privadas nacidas de la división y concesión de la estatal Servicios Eléctricos del Gran Buenos Aires (SEGBA).
 El proceso de reestructuración apuntó a erradicar los recurrentes cortes rotativos y el déficit operativo crónico de la empresa estatal, transfiriendo las redes de distribución a consorcios de capitales franceses, chilenos y locales.
 ¿Mejoró la calidad del suministro eléctrico tras la privatización de 1992? Opiná abajo.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -13652,7 +13652,7 @@
           <t>El 1 de enero de 1992 comenzó a circular formalmente el Peso ($), el actual signo monetario de la República Argentina. Tras dos años de hiperinflación y el fracaso terminal del Austral, Domingo Cavallo dispuso quitar cuatro ceros a la moneda desvalorizada.
 Cada nuevo peso equivalía exactamente a 10.000 australes y a un dólar estadounidense depositado en las bóvedas del Banco Central. Nacía una década de estabilidad cambiaria y de precios que transformó el consumo y el crédito de los argentinos.
 ¿Recordás cuál fue el primer billete de la nueva convertibilidad que tuviste en tus manos? Contanos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -13734,7 +13734,7 @@
           <t>En julio de 1935, el Congreso Nacional fue escenario de la jornada más dramática de la historia política argentina. El senador demócrata progresista Lisandro de la Torre presentó una exhaustiva investigación que demostraba la evasión tributaria y el monopolio de los frigoríficos anglo-norteamericanos.
 Los ministros Luis Duhau y Federico Pinedo fueron interpelados en un clima de tensión extrema. En pleno recinto de la Cámara Alta, un sicario vinculado al oficialismo disparó contra De la Torre, pero las balas impactaron en su compañero de bancada Enzo Bordabehere, quien murió en el acto.
 ¿Conocías el trágico desenlace del debate sobre el monopolio de la carne en los años 30? Te leemos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -13816,7 +13816,7 @@
           <t>En agosto de 1962, durante el gobierno de José María Guido tras el derrocamiento de Frondizi, la tesorería pública colapsó por falta de fondos. El ministro de Economía Álvaro Alsogaray tomó una medida extrema: emitir los bonos 'Empréstito 9 de Julio'.
 Los empleados estatales, docentes y jubilados cobraron sus salarios atrasados con estos títulos de deuda pública de suscripción forzosa, viéndose obligados a venderlos en la Bolsa de Comercio con quitas del 30% al 40% para comprar alimentos.
 ¿Recordabas cuando el Estado argentino pagaba sueldos enteros con bonos de deuda? Te leemos en comentarios.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>
@@ -13898,7 +13898,7 @@
           <t>En la noche del 27 de octubre de 2019, mientras se confirmaba la victoria de Alberto Fernández en primera vuelta presidencial, el directorio del Banco Central presidido por Guido Sandleris emitió la Comunicación 'A' 6815 a la medianoche.
 Para evitar que las reservas líquidas se extinguieran antes del traspaso de mando del 10 de diciembre, el cupo de compra de dólares para atesoramiento se desplomó de 10.000 dólares a un estricto límite de 200 dólares por mes por cuenta bancaria, consagrando el regreso del cepo cambiario duro.
 ¿Recordás qué hiciste con tus ahorros los días posteriores a la reimposición del cepo? Contanos.
-📺 Encontrá el documental y análisis completo en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
+📺 Más sobre historia económica argentina en nuestro canal de YouTube: @hablemosdeeco (link en el perfil).
 #HistoriaEconomica #EconomiaArgentina #HablemosDeEconomia</t>
         </is>
       </c>

</xml_diff>

<commit_message>
chore(auditoria): sincronizar excel con post 10 publicado
</commit_message>
<xml_diff>
--- a/auditoria_datos_hde.xlsx
+++ b/auditoria_datos_hde.xlsx
@@ -1368,9 +1368,9 @@
       <c r="A11" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore(auditoria): sincronizar excel con 24 posts publicados al 28-oct
</commit_message>
<xml_diff>
--- a/auditoria_datos_hde.xlsx
+++ b/auditoria_datos_hde.xlsx
@@ -1450,9 +1450,9 @@
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1532,9 +1532,9 @@
       <c r="A13" s="9" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -1614,9 +1614,9 @@
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1696,9 +1696,9 @@
       <c r="A15" s="9" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -1778,9 +1778,9 @@
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -1860,9 +1860,9 @@
       <c r="A17" s="9" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -1942,9 +1942,9 @@
       <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -2024,9 +2024,9 @@
       <c r="A19" s="9" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -2106,9 +2106,9 @@
       <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -2926,9 +2926,9 @@
       <c r="A30" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
@@ -10880,9 +10880,9 @@
       <c r="A127" s="9" t="n">
         <v>126</v>
       </c>
-      <c r="B127" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="B127" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
         </is>
       </c>
       <c r="C127" s="4" t="inlineStr">
@@ -11454,9 +11454,9 @@
       <c r="A134" s="2" t="n">
         <v>133</v>
       </c>
-      <c r="B134" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="B134" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
         </is>
       </c>
       <c r="C134" s="4" t="inlineStr">
@@ -13832,9 +13832,9 @@
       <c r="A163" s="9" t="n">
         <v>162</v>
       </c>
-      <c r="B163" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="B163" s="3" t="inlineStr">
+        <is>
+          <t>SI</t>
         </is>
       </c>
       <c r="C163" s="4" t="inlineStr">

</xml_diff>